<commit_message>
#251219 fix: fixed global settings
</commit_message>
<xml_diff>
--- a/files/email-list.xlsx
+++ b/files/email-list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koray.zorlu\projects\arierp\arierp_backend\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7B50FC9-941C-43C9-962F-D7CC1EB6A4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D703416-DCCA-4ED1-A3D0-8ACB83F5C8D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -221,7 +221,8 @@
   <dimension ref="A1:F248"/>
   <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="25.90625" customWidth="1"/>
+    <col min="1" max="1" width="51.1796875" customWidth="1"/>
+    <col min="2" max="2" width="25.90625" customWidth="1"/>
     <col min="3" max="3" width="35.54296875" customWidth="1"/>
     <col min="4" max="4" width="12.453125" customWidth="1"/>
   </cols>
@@ -257,7 +258,7 @@
       <c r="F3" s="1"/>
     </row>
     <row r="4" spans="1:6" ht="13" x14ac:dyDescent="0.3">
-      <c r="A4" s="1"/>
+      <c r="A4" s="2"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -265,7 +266,7 @@
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:6" ht="13" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
+      <c r="A5" s="2"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>

</xml_diff>